<commit_message>
data(eur): all refresh 2026-09-09T12:23Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
+++ b/logs/eur/raw/finanzagentur_emissionsergebnisse_aktuell_en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="197" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="198" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -681,6 +681,9 @@
   </si>
   <si>
     <t>86</t>
+  </si>
+  <si>
+    <t>87</t>
   </si>
   <si>
     <t>Sum:</t>
@@ -1124,7 +1127,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S166"/>
+  <dimension ref="A1:S167"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="3.637802" bestFit="1" customWidth="1"/>
@@ -9594,108 +9597,167 @@
       </c>
     </row>
     <row r="155" spans="1:19">
-      <c r="A155" s="50" t="s">
+      <c r="A155" s="36" t="s">
         <v>183</v>
       </c>
-      <c r="B155" s="48"/>
-      <c r="C155" s="48"/>
-      <c r="D155" s="48"/>
-      <c r="E155" s="48"/>
-      <c r="F155" s="48"/>
-      <c r="G155" s="49"/>
-      <c r="H155" s="52">
-        <v>382500</v>
-      </c>
-      <c r="I155" s="51"/>
-      <c r="J155" s="51"/>
-      <c r="K155" s="52">
-        <v>520459</v>
-      </c>
-      <c r="L155" s="52">
-        <v>304864</v>
-      </c>
-      <c r="M155" s="52">
-        <v>215595</v>
-      </c>
-      <c r="N155" s="53">
-        <v>301008.44</v>
-      </c>
-      <c r="O155" s="47"/>
-      <c r="P155" s="48"/>
-      <c r="Q155" s="48"/>
-      <c r="R155" s="49"/>
-      <c r="S155" s="54">
-        <v>1.727382272071</v>
-      </c>
-    </row>
-    <row r="156" spans="1:1" customHeight="1" ht="19.500000">
-      <c r="A156" s="21" t="s">
+      <c r="B155" s="37">
+        <v>46274</v>
+      </c>
+      <c r="C155" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="D155" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E155" s="45">
+        <v>0.03</v>
+      </c>
+      <c r="F155" s="37">
+        <v>49902</v>
+      </c>
+      <c r="G155" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="H155" s="39">
+        <v>5500</v>
+      </c>
+      <c r="I155" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="J155" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="K155" s="39">
+        <v>6186</v>
+      </c>
+      <c r="L155" s="39">
+        <v>4095</v>
+      </c>
+      <c r="M155" s="39">
+        <v>2091</v>
+      </c>
+      <c r="N155" s="40">
+        <v>4200.99</v>
+      </c>
+      <c r="O155" s="41">
+        <v>96.72</v>
+      </c>
+      <c r="P155" s="40">
+        <v>96.73</v>
+      </c>
+      <c r="Q155" s="40">
+        <v>3.39</v>
+      </c>
+      <c r="R155" s="40">
+        <v>1299.01</v>
+      </c>
+      <c r="S155" s="44">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="156" spans="1:19">
+      <c r="A156" s="50" t="s">
+        <v>184</v>
+      </c>
+      <c r="B156" s="48"/>
+      <c r="C156" s="48"/>
+      <c r="D156" s="48"/>
+      <c r="E156" s="48"/>
+      <c r="F156" s="48"/>
+      <c r="G156" s="49"/>
+      <c r="H156" s="52">
+        <v>388000</v>
+      </c>
+      <c r="I156" s="51"/>
+      <c r="J156" s="51"/>
+      <c r="K156" s="52">
+        <v>526645</v>
+      </c>
+      <c r="L156" s="52">
+        <v>308959</v>
+      </c>
+      <c r="M156" s="52">
+        <v>217686</v>
+      </c>
+      <c r="N156" s="53">
+        <v>305209.43</v>
+      </c>
+      <c r="O156" s="47"/>
+      <c r="P156" s="48"/>
+      <c r="Q156" s="48"/>
+      <c r="R156" s="49"/>
+      <c r="S156" s="54">
+        <v>1.724252517361</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" customHeight="1" ht="19.500000">
+      <c r="A157" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:2">
-      <c r="A157" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B157" s="22" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="158" spans="1:1">
+    <row r="158" spans="1:2">
       <c r="A158" s="22" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="159" spans="1:2">
-      <c r="A159" s="23" t="s">
+      <c r="B158" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="B159" s="26" t="s">
+    </row>
+    <row r="159" spans="1:1">
+      <c r="A159" s="22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="23" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="161" spans="1:2">
-      <c r="A161" s="23" t="s">
+      <c r="B160" s="26" t="s">
         <v>187</v>
-      </c>
-      <c r="B161" s="22" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="B162" s="22" t="s">
         <v>189</v>
-      </c>
-      <c r="B162" s="22" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="B163" s="22" t="s">
         <v>191</v>
-      </c>
-      <c r="B163" s="22" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B164" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="B164" s="22" t="s">
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="23" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="165" spans="1:2">
-      <c r="A165" s="24" t="s">
+      <c r="B165" s="22" t="s">
         <v>195</v>
       </c>
-      <c r="B165" s="22" t="s">
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="24" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="166" spans="1:1">
-      <c r="A166" s="25" t="s">
+      <c r="B166" s="22" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1">
+      <c r="A167" s="25" t="s">
         <v>1</v>
       </c>
     </row>
@@ -9705,16 +9767,16 @@
     <mergeCell ref="A6:S6"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="C8:C11"/>
-    <mergeCell ref="A155:G155"/>
-    <mergeCell ref="O155:R155"/>
-    <mergeCell ref="B157:R157"/>
-    <mergeCell ref="A159:A160"/>
-    <mergeCell ref="B159:R160"/>
-    <mergeCell ref="B161:R161"/>
+    <mergeCell ref="A156:G156"/>
+    <mergeCell ref="O156:R156"/>
+    <mergeCell ref="B158:R158"/>
+    <mergeCell ref="A160:A161"/>
+    <mergeCell ref="B160:R161"/>
     <mergeCell ref="B162:R162"/>
     <mergeCell ref="B163:R163"/>
     <mergeCell ref="B164:R164"/>
     <mergeCell ref="B165:R165"/>
+    <mergeCell ref="B166:R166"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>